<commit_message>
Update data and UI for April 26, 2026 - Add growth percentage to total line chart
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -535,13 +535,13 @@
         <v>150469</v>
       </c>
       <c r="L2" t="n">
-        <v>42350</v>
+        <v>48992</v>
       </c>
       <c r="M2" t="n">
-        <v>8740</v>
+        <v>10702</v>
       </c>
       <c r="N2" t="n">
-        <v>33610</v>
+        <v>38290</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>81428</v>
       </c>
       <c r="L3" t="n">
-        <v>70260</v>
+        <v>81591</v>
       </c>
       <c r="M3" t="n">
-        <v>26121</v>
+        <v>32215</v>
       </c>
       <c r="N3" t="n">
-        <v>44139</v>
+        <v>49376</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +623,13 @@
         <v>18713</v>
       </c>
       <c r="L4" t="n">
-        <v>12792</v>
+        <v>14746</v>
       </c>
       <c r="M4" t="n">
-        <v>2155</v>
+        <v>2571</v>
       </c>
       <c r="N4" t="n">
-        <v>10637</v>
+        <v>12175</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         <v>42408</v>
       </c>
       <c r="L5" t="n">
-        <v>16345</v>
+        <v>18534</v>
       </c>
       <c r="M5" t="n">
-        <v>4236</v>
+        <v>5012</v>
       </c>
       <c r="N5" t="n">
-        <v>12109</v>
+        <v>13522</v>
       </c>
     </row>
     <row r="6">
@@ -711,13 +711,13 @@
         <v>117439</v>
       </c>
       <c r="L6" t="n">
-        <v>46160</v>
+        <v>52495</v>
       </c>
       <c r="M6" t="n">
-        <v>10319</v>
+        <v>12483</v>
       </c>
       <c r="N6" t="n">
-        <v>35841</v>
+        <v>40012</v>
       </c>
     </row>
     <row r="7">
@@ -755,13 +755,13 @@
         <v>19076</v>
       </c>
       <c r="L7" t="n">
-        <v>6328</v>
+        <v>7502</v>
       </c>
       <c r="M7" t="n">
-        <v>902</v>
+        <v>1170</v>
       </c>
       <c r="N7" t="n">
-        <v>5426</v>
+        <v>6332</v>
       </c>
     </row>
     <row r="8">
@@ -799,13 +799,13 @@
         <v>83014</v>
       </c>
       <c r="L8" t="n">
-        <v>44892</v>
+        <v>50439</v>
       </c>
       <c r="M8" t="n">
-        <v>9194</v>
+        <v>10908</v>
       </c>
       <c r="N8" t="n">
-        <v>35698</v>
+        <v>39531</v>
       </c>
     </row>
     <row r="9">
@@ -843,13 +843,13 @@
         <v>65107</v>
       </c>
       <c r="L9" t="n">
-        <v>32932</v>
+        <v>37574</v>
       </c>
       <c r="M9" t="n">
-        <v>9499</v>
+        <v>11434</v>
       </c>
       <c r="N9" t="n">
-        <v>23433</v>
+        <v>26140</v>
       </c>
     </row>
     <row r="10">
@@ -887,13 +887,13 @@
         <v>151451</v>
       </c>
       <c r="L10" t="n">
-        <v>61307</v>
+        <v>70644</v>
       </c>
       <c r="M10" t="n">
-        <v>19113</v>
+        <v>23253</v>
       </c>
       <c r="N10" t="n">
-        <v>42194</v>
+        <v>47391</v>
       </c>
     </row>
     <row r="11">
@@ -931,13 +931,13 @@
         <v>127517</v>
       </c>
       <c r="L11" t="n">
-        <v>41698</v>
+        <v>48032</v>
       </c>
       <c r="M11" t="n">
-        <v>9421</v>
+        <v>11747</v>
       </c>
       <c r="N11" t="n">
-        <v>32277</v>
+        <v>36285</v>
       </c>
     </row>
     <row r="12">
@@ -975,13 +975,13 @@
         <v>122266</v>
       </c>
       <c r="L12" t="n">
-        <v>51315</v>
+        <v>59595</v>
       </c>
       <c r="M12" t="n">
-        <v>8936</v>
+        <v>10920</v>
       </c>
       <c r="N12" t="n">
-        <v>42379</v>
+        <v>48675</v>
       </c>
     </row>
     <row r="13">
@@ -1019,13 +1019,13 @@
         <v>399425</v>
       </c>
       <c r="L13" t="n">
-        <v>133518</v>
+        <v>156005</v>
       </c>
       <c r="M13" t="n">
-        <v>67237</v>
+        <v>80881</v>
       </c>
       <c r="N13" t="n">
-        <v>66281</v>
+        <v>75124</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         <v>274795</v>
       </c>
       <c r="L14" t="n">
-        <v>153137</v>
+        <v>176541</v>
       </c>
       <c r="M14" t="n">
-        <v>71410</v>
+        <v>86086</v>
       </c>
       <c r="N14" t="n">
-        <v>81727</v>
+        <v>90455</v>
       </c>
     </row>
     <row r="15">
@@ -1107,13 +1107,13 @@
         <v>80530</v>
       </c>
       <c r="L15" t="n">
-        <v>46045</v>
+        <v>55674</v>
       </c>
       <c r="M15" t="n">
-        <v>15631</v>
+        <v>19759</v>
       </c>
       <c r="N15" t="n">
-        <v>30414</v>
+        <v>35915</v>
       </c>
     </row>
     <row r="16">
@@ -1151,13 +1151,13 @@
         <v>15975</v>
       </c>
       <c r="L16" t="n">
-        <v>35414</v>
+        <v>39931</v>
       </c>
       <c r="M16" t="n">
-        <v>4943</v>
+        <v>5958</v>
       </c>
       <c r="N16" t="n">
-        <v>30471</v>
+        <v>33973</v>
       </c>
     </row>
     <row r="17">
@@ -1195,13 +1195,13 @@
         <v>26564</v>
       </c>
       <c r="L17" t="n">
-        <v>17192</v>
+        <v>19523</v>
       </c>
       <c r="M17" t="n">
-        <v>4505</v>
+        <v>5524</v>
       </c>
       <c r="N17" t="n">
-        <v>12687</v>
+        <v>13999</v>
       </c>
     </row>
     <row r="18">
@@ -1239,13 +1239,13 @@
         <v>66764</v>
       </c>
       <c r="L18" t="n">
-        <v>44687</v>
+        <v>53656</v>
       </c>
       <c r="M18" t="n">
-        <v>12537</v>
+        <v>15881</v>
       </c>
       <c r="N18" t="n">
-        <v>32150</v>
+        <v>37775</v>
       </c>
     </row>
     <row r="19">
@@ -1283,13 +1283,13 @@
         <v>55231</v>
       </c>
       <c r="L19" t="n">
-        <v>29959</v>
+        <v>33416</v>
       </c>
       <c r="M19" t="n">
-        <v>7729</v>
+        <v>9335</v>
       </c>
       <c r="N19" t="n">
-        <v>22230</v>
+        <v>24081</v>
       </c>
     </row>
     <row r="20">
@@ -1327,13 +1327,13 @@
         <v>58737</v>
       </c>
       <c r="L20" t="n">
-        <v>24513</v>
+        <v>28248</v>
       </c>
       <c r="M20" t="n">
-        <v>6226</v>
+        <v>7554</v>
       </c>
       <c r="N20" t="n">
-        <v>18287</v>
+        <v>20694</v>
       </c>
     </row>
     <row r="21">
@@ -1371,13 +1371,13 @@
         <v>24382</v>
       </c>
       <c r="L21" t="n">
-        <v>8347</v>
+        <v>10815</v>
       </c>
       <c r="M21" t="n">
-        <v>2130</v>
+        <v>2949</v>
       </c>
       <c r="N21" t="n">
-        <v>6217</v>
+        <v>7866</v>
       </c>
     </row>
     <row r="22">
@@ -1415,13 +1415,13 @@
         <v>152229</v>
       </c>
       <c r="L22" t="n">
-        <v>51459</v>
+        <v>58868</v>
       </c>
       <c r="M22" t="n">
-        <v>12983</v>
+        <v>15702</v>
       </c>
       <c r="N22" t="n">
-        <v>38476</v>
+        <v>43166</v>
       </c>
     </row>
     <row r="23">
@@ -1459,13 +1459,13 @@
         <v>40867</v>
       </c>
       <c r="L23" t="n">
-        <v>19168</v>
+        <v>21833</v>
       </c>
       <c r="M23" t="n">
-        <v>4317</v>
+        <v>5102</v>
       </c>
       <c r="N23" t="n">
-        <v>14851</v>
+        <v>16731</v>
       </c>
     </row>
     <row r="24">
@@ -1503,13 +1503,13 @@
         <v>88798</v>
       </c>
       <c r="L24" t="n">
-        <v>61172</v>
+        <v>70489</v>
       </c>
       <c r="M24" t="n">
-        <v>12732</v>
+        <v>15718</v>
       </c>
       <c r="N24" t="n">
-        <v>48440</v>
+        <v>54771</v>
       </c>
     </row>
     <row r="25">
@@ -1547,13 +1547,13 @@
         <v>86600</v>
       </c>
       <c r="L25" t="n">
-        <v>38791</v>
+        <v>47096</v>
       </c>
       <c r="M25" t="n">
-        <v>12737</v>
+        <v>16203</v>
       </c>
       <c r="N25" t="n">
-        <v>26054</v>
+        <v>30893</v>
       </c>
     </row>
     <row r="26">
@@ -1591,13 +1591,13 @@
         <v>95605</v>
       </c>
       <c r="L26" t="n">
-        <v>60203</v>
+        <v>70975</v>
       </c>
       <c r="M26" t="n">
-        <v>18146</v>
+        <v>23108</v>
       </c>
       <c r="N26" t="n">
-        <v>42057</v>
+        <v>47867</v>
       </c>
     </row>
     <row r="27">
@@ -1635,13 +1635,13 @@
         <v>35197</v>
       </c>
       <c r="L27" t="n">
-        <v>22220</v>
+        <v>25830</v>
       </c>
       <c r="M27" t="n">
-        <v>6106</v>
+        <v>7358</v>
       </c>
       <c r="N27" t="n">
-        <v>16114</v>
+        <v>18472</v>
       </c>
     </row>
     <row r="28">
@@ -1679,13 +1679,13 @@
         <v>52800</v>
       </c>
       <c r="L28" t="n">
-        <v>34416</v>
+        <v>38075</v>
       </c>
       <c r="M28" t="n">
-        <v>5186</v>
+        <v>6206</v>
       </c>
       <c r="N28" t="n">
-        <v>29230</v>
+        <v>31869</v>
       </c>
     </row>
     <row r="29">
@@ -1723,13 +1723,13 @@
         <v>34093</v>
       </c>
       <c r="L29" t="n">
-        <v>19779</v>
+        <v>23465</v>
       </c>
       <c r="M29" t="n">
-        <v>3167</v>
+        <v>3946</v>
       </c>
       <c r="N29" t="n">
-        <v>16612</v>
+        <v>19519</v>
       </c>
     </row>
     <row r="30">
@@ -1767,13 +1767,13 @@
         <v>59519</v>
       </c>
       <c r="L30" t="n">
-        <v>20885</v>
+        <v>23391</v>
       </c>
       <c r="M30" t="n">
-        <v>3529</v>
+        <v>4215</v>
       </c>
       <c r="N30" t="n">
-        <v>17356</v>
+        <v>19176</v>
       </c>
     </row>
     <row r="31">
@@ -1811,13 +1811,13 @@
         <v>111215</v>
       </c>
       <c r="L31" t="n">
-        <v>41055</v>
+        <v>49528</v>
       </c>
       <c r="M31" t="n">
-        <v>9089</v>
+        <v>11623</v>
       </c>
       <c r="N31" t="n">
-        <v>31966</v>
+        <v>37905</v>
       </c>
     </row>
     <row r="32">
@@ -1855,13 +1855,13 @@
         <v>135620</v>
       </c>
       <c r="L32" t="n">
-        <v>45519</v>
+        <v>52818</v>
       </c>
       <c r="M32" t="n">
-        <v>10745</v>
+        <v>13326</v>
       </c>
       <c r="N32" t="n">
-        <v>34774</v>
+        <v>39492</v>
       </c>
     </row>
     <row r="33">
@@ -1899,13 +1899,13 @@
         <v>46108</v>
       </c>
       <c r="L33" t="n">
-        <v>31495</v>
+        <v>36461</v>
       </c>
       <c r="M33" t="n">
-        <v>9869</v>
+        <v>12197</v>
       </c>
       <c r="N33" t="n">
-        <v>21626</v>
+        <v>24264</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>74035</v>
       </c>
       <c r="L34" t="n">
-        <v>33050</v>
+        <v>37860</v>
       </c>
       <c r="M34" t="n">
-        <v>6619</v>
+        <v>7928</v>
       </c>
       <c r="N34" t="n">
-        <v>26431</v>
+        <v>29932</v>
       </c>
     </row>
     <row r="35">
@@ -1987,13 +1987,13 @@
         <v>134411</v>
       </c>
       <c r="L35" t="n">
-        <v>44430</v>
+        <v>50347</v>
       </c>
       <c r="M35" t="n">
-        <v>8181</v>
+        <v>10212</v>
       </c>
       <c r="N35" t="n">
-        <v>36249</v>
+        <v>40135</v>
       </c>
     </row>
     <row r="36">
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>34235</v>
+        <v>39307</v>
       </c>
       <c r="M36" t="n">
-        <v>5872</v>
+        <v>7188</v>
       </c>
       <c r="N36" t="n">
-        <v>28363</v>
+        <v>32119</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>54545</v>
+        <v>62713</v>
       </c>
       <c r="M37" t="n">
-        <v>17052</v>
+        <v>21119</v>
       </c>
       <c r="N37" t="n">
-        <v>37493</v>
+        <v>41594</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>11910</v>
+        <v>13683</v>
       </c>
       <c r="M38" t="n">
-        <v>1896</v>
+        <v>2257</v>
       </c>
       <c r="N38" t="n">
-        <v>10014</v>
+        <v>11426</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>13002</v>
+        <v>14649</v>
       </c>
       <c r="M39" t="n">
-        <v>2635</v>
+        <v>3084</v>
       </c>
       <c r="N39" t="n">
-        <v>10367</v>
+        <v>11565</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>36929</v>
+        <v>41630</v>
       </c>
       <c r="M40" t="n">
-        <v>6209</v>
+        <v>7535</v>
       </c>
       <c r="N40" t="n">
-        <v>30720</v>
+        <v>34095</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>5329</v>
+        <v>6291</v>
       </c>
       <c r="M41" t="n">
-        <v>688</v>
+        <v>894</v>
       </c>
       <c r="N41" t="n">
-        <v>4641</v>
+        <v>5397</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>39829</v>
+        <v>44589</v>
       </c>
       <c r="M42" t="n">
-        <v>7396</v>
+        <v>8771</v>
       </c>
       <c r="N42" t="n">
-        <v>32433</v>
+        <v>35818</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>27258</v>
+        <v>30827</v>
       </c>
       <c r="M43" t="n">
-        <v>6058</v>
+        <v>7265</v>
       </c>
       <c r="N43" t="n">
-        <v>21200</v>
+        <v>23562</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>50407</v>
+        <v>57630</v>
       </c>
       <c r="M44" t="n">
-        <v>12857</v>
+        <v>15642</v>
       </c>
       <c r="N44" t="n">
-        <v>37550</v>
+        <v>41988</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>34299</v>
+        <v>39346</v>
       </c>
       <c r="M45" t="n">
-        <v>6462</v>
+        <v>8167</v>
       </c>
       <c r="N45" t="n">
-        <v>27837</v>
+        <v>31179</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>45315</v>
+        <v>52371</v>
       </c>
       <c r="M46" t="n">
-        <v>6879</v>
+        <v>8403</v>
       </c>
       <c r="N46" t="n">
-        <v>38436</v>
+        <v>43968</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>85359</v>
+        <v>99207</v>
       </c>
       <c r="M47" t="n">
-        <v>35107</v>
+        <v>42350</v>
       </c>
       <c r="N47" t="n">
-        <v>50252</v>
+        <v>56857</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>88894</v>
+        <v>101644</v>
       </c>
       <c r="M48" t="n">
-        <v>34040</v>
+        <v>41171</v>
       </c>
       <c r="N48" t="n">
-        <v>54854</v>
+        <v>60473</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>31779</v>
+        <v>38308</v>
       </c>
       <c r="M49" t="n">
-        <v>8781</v>
+        <v>11280</v>
       </c>
       <c r="N49" t="n">
-        <v>22998</v>
+        <v>27028</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>30456</v>
+        <v>34088</v>
       </c>
       <c r="M50" t="n">
-        <v>3575</v>
+        <v>4266</v>
       </c>
       <c r="N50" t="n">
-        <v>26881</v>
+        <v>29822</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>14080</v>
+        <v>15822</v>
       </c>
       <c r="M51" t="n">
-        <v>2876</v>
+        <v>3532</v>
       </c>
       <c r="N51" t="n">
-        <v>11204</v>
+        <v>12290</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>33343</v>
+        <v>39827</v>
       </c>
       <c r="M52" t="n">
-        <v>7449</v>
+        <v>9572</v>
       </c>
       <c r="N52" t="n">
-        <v>25894</v>
+        <v>30255</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>26204</v>
+        <v>29069</v>
       </c>
       <c r="M53" t="n">
-        <v>5877</v>
+        <v>7115</v>
       </c>
       <c r="N53" t="n">
-        <v>20327</v>
+        <v>21954</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>21467</v>
+        <v>24610</v>
       </c>
       <c r="M54" t="n">
-        <v>5156</v>
+        <v>6247</v>
       </c>
       <c r="N54" t="n">
-        <v>16311</v>
+        <v>18363</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>6979</v>
+        <v>8997</v>
       </c>
       <c r="M55" t="n">
-        <v>1667</v>
+        <v>2320</v>
       </c>
       <c r="N55" t="n">
-        <v>5312</v>
+        <v>6677</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>45324</v>
+        <v>51552</v>
       </c>
       <c r="M56" t="n">
-        <v>10165</v>
+        <v>12265</v>
       </c>
       <c r="N56" t="n">
-        <v>35159</v>
+        <v>39287</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>17010</v>
+        <v>19325</v>
       </c>
       <c r="M57" t="n">
-        <v>3607</v>
+        <v>4256</v>
       </c>
       <c r="N57" t="n">
-        <v>13403</v>
+        <v>15069</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>52396</v>
+        <v>59970</v>
       </c>
       <c r="M58" t="n">
-        <v>9174</v>
+        <v>11281</v>
       </c>
       <c r="N58" t="n">
-        <v>43222</v>
+        <v>48689</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>27799</v>
+        <v>33530</v>
       </c>
       <c r="M59" t="n">
-        <v>7132</v>
+        <v>9228</v>
       </c>
       <c r="N59" t="n">
-        <v>20667</v>
+        <v>24302</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>48520</v>
+        <v>56818</v>
       </c>
       <c r="M60" t="n">
-        <v>12624</v>
+        <v>16179</v>
       </c>
       <c r="N60" t="n">
-        <v>35896</v>
+        <v>40639</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>16795</v>
+        <v>19462</v>
       </c>
       <c r="M61" t="n">
-        <v>3967</v>
+        <v>4769</v>
       </c>
       <c r="N61" t="n">
-        <v>12828</v>
+        <v>14693</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>31423</v>
+        <v>34589</v>
       </c>
       <c r="M62" t="n">
-        <v>4039</v>
+        <v>4821</v>
       </c>
       <c r="N62" t="n">
-        <v>27384</v>
+        <v>29768</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>16687</v>
+        <v>19635</v>
       </c>
       <c r="M63" t="n">
-        <v>2172</v>
+        <v>2720</v>
       </c>
       <c r="N63" t="n">
-        <v>14515</v>
+        <v>16915</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>18472</v>
+        <v>20549</v>
       </c>
       <c r="M64" t="n">
-        <v>2941</v>
+        <v>3479</v>
       </c>
       <c r="N64" t="n">
-        <v>15531</v>
+        <v>17070</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>33195</v>
+        <v>39845</v>
       </c>
       <c r="M65" t="n">
-        <v>5992</v>
+        <v>7766</v>
       </c>
       <c r="N65" t="n">
-        <v>27203</v>
+        <v>32079</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>35481</v>
+        <v>40947</v>
       </c>
       <c r="M66" t="n">
-        <v>6547</v>
+        <v>8182</v>
       </c>
       <c r="N66" t="n">
-        <v>28934</v>
+        <v>32765</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>26935</v>
+        <v>31014</v>
       </c>
       <c r="M67" t="n">
-        <v>7367</v>
+        <v>9149</v>
       </c>
       <c r="N67" t="n">
-        <v>19568</v>
+        <v>21865</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>29337</v>
+        <v>33485</v>
       </c>
       <c r="M68" t="n">
-        <v>5624</v>
+        <v>6719</v>
       </c>
       <c r="N68" t="n">
-        <v>23713</v>
+        <v>26766</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>37394</v>
+        <v>42102</v>
       </c>
       <c r="M69" t="n">
-        <v>5404</v>
+        <v>6797</v>
       </c>
       <c r="N69" t="n">
-        <v>31990</v>
+        <v>35305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboard data for 2026-04-27
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -535,13 +535,13 @@
         <v>150469</v>
       </c>
       <c r="L2" t="n">
-        <v>48992</v>
+        <v>58428</v>
       </c>
       <c r="M2" t="n">
-        <v>10702</v>
+        <v>13110</v>
       </c>
       <c r="N2" t="n">
-        <v>38290</v>
+        <v>45318</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>81428</v>
       </c>
       <c r="L3" t="n">
-        <v>81591</v>
+        <v>95067</v>
       </c>
       <c r="M3" t="n">
-        <v>32215</v>
+        <v>38520</v>
       </c>
       <c r="N3" t="n">
-        <v>49376</v>
+        <v>56547</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +623,13 @@
         <v>18713</v>
       </c>
       <c r="L4" t="n">
-        <v>14746</v>
+        <v>16985</v>
       </c>
       <c r="M4" t="n">
-        <v>2571</v>
+        <v>3063</v>
       </c>
       <c r="N4" t="n">
-        <v>12175</v>
+        <v>13922</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         <v>42408</v>
       </c>
       <c r="L5" t="n">
-        <v>18534</v>
+        <v>21521</v>
       </c>
       <c r="M5" t="n">
-        <v>5012</v>
+        <v>5893</v>
       </c>
       <c r="N5" t="n">
-        <v>13522</v>
+        <v>15628</v>
       </c>
     </row>
     <row r="6">
@@ -711,13 +711,13 @@
         <v>117439</v>
       </c>
       <c r="L6" t="n">
-        <v>52495</v>
+        <v>61859</v>
       </c>
       <c r="M6" t="n">
-        <v>12483</v>
+        <v>14733</v>
       </c>
       <c r="N6" t="n">
-        <v>40012</v>
+        <v>47126</v>
       </c>
     </row>
     <row r="7">
@@ -755,13 +755,13 @@
         <v>19076</v>
       </c>
       <c r="L7" t="n">
-        <v>7502</v>
+        <v>8872</v>
       </c>
       <c r="M7" t="n">
-        <v>1170</v>
+        <v>1444</v>
       </c>
       <c r="N7" t="n">
-        <v>6332</v>
+        <v>7428</v>
       </c>
     </row>
     <row r="8">
@@ -799,13 +799,13 @@
         <v>83014</v>
       </c>
       <c r="L8" t="n">
-        <v>50439</v>
+        <v>57942</v>
       </c>
       <c r="M8" t="n">
-        <v>10908</v>
+        <v>12877</v>
       </c>
       <c r="N8" t="n">
-        <v>39531</v>
+        <v>45065</v>
       </c>
     </row>
     <row r="9">
@@ -843,13 +843,13 @@
         <v>65107</v>
       </c>
       <c r="L9" t="n">
-        <v>37574</v>
+        <v>43797</v>
       </c>
       <c r="M9" t="n">
-        <v>11434</v>
+        <v>13283</v>
       </c>
       <c r="N9" t="n">
-        <v>26140</v>
+        <v>30514</v>
       </c>
     </row>
     <row r="10">
@@ -887,13 +887,13 @@
         <v>151451</v>
       </c>
       <c r="L10" t="n">
-        <v>70644</v>
+        <v>81959</v>
       </c>
       <c r="M10" t="n">
-        <v>23253</v>
+        <v>27452</v>
       </c>
       <c r="N10" t="n">
-        <v>47391</v>
+        <v>54507</v>
       </c>
     </row>
     <row r="11">
@@ -931,13 +931,13 @@
         <v>127517</v>
       </c>
       <c r="L11" t="n">
-        <v>48032</v>
+        <v>57074</v>
       </c>
       <c r="M11" t="n">
-        <v>11747</v>
+        <v>14202</v>
       </c>
       <c r="N11" t="n">
-        <v>36285</v>
+        <v>42872</v>
       </c>
     </row>
     <row r="12">
@@ -975,13 +975,13 @@
         <v>122266</v>
       </c>
       <c r="L12" t="n">
-        <v>59595</v>
+        <v>69826</v>
       </c>
       <c r="M12" t="n">
-        <v>10920</v>
+        <v>13246</v>
       </c>
       <c r="N12" t="n">
-        <v>48675</v>
+        <v>56580</v>
       </c>
     </row>
     <row r="13">
@@ -1019,13 +1019,13 @@
         <v>399425</v>
       </c>
       <c r="L13" t="n">
-        <v>156005</v>
+        <v>183303</v>
       </c>
       <c r="M13" t="n">
-        <v>80881</v>
+        <v>93836</v>
       </c>
       <c r="N13" t="n">
-        <v>75124</v>
+        <v>89467</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         <v>274795</v>
       </c>
       <c r="L14" t="n">
-        <v>176541</v>
+        <v>204790</v>
       </c>
       <c r="M14" t="n">
-        <v>86086</v>
+        <v>100981</v>
       </c>
       <c r="N14" t="n">
-        <v>90455</v>
+        <v>103809</v>
       </c>
     </row>
     <row r="15">
@@ -1107,13 +1107,13 @@
         <v>80530</v>
       </c>
       <c r="L15" t="n">
-        <v>55674</v>
+        <v>65401</v>
       </c>
       <c r="M15" t="n">
-        <v>19759</v>
+        <v>23582</v>
       </c>
       <c r="N15" t="n">
-        <v>35915</v>
+        <v>41819</v>
       </c>
     </row>
     <row r="16">
@@ -1151,13 +1151,13 @@
         <v>15975</v>
       </c>
       <c r="L16" t="n">
-        <v>39931</v>
+        <v>45918</v>
       </c>
       <c r="M16" t="n">
-        <v>5958</v>
+        <v>7006</v>
       </c>
       <c r="N16" t="n">
-        <v>33973</v>
+        <v>38912</v>
       </c>
     </row>
     <row r="17">
@@ -1195,13 +1195,13 @@
         <v>26564</v>
       </c>
       <c r="L17" t="n">
-        <v>19523</v>
+        <v>23028</v>
       </c>
       <c r="M17" t="n">
-        <v>5524</v>
+        <v>6581</v>
       </c>
       <c r="N17" t="n">
-        <v>13999</v>
+        <v>16447</v>
       </c>
     </row>
     <row r="18">
@@ -1239,13 +1239,13 @@
         <v>66764</v>
       </c>
       <c r="L18" t="n">
-        <v>53656</v>
+        <v>62289</v>
       </c>
       <c r="M18" t="n">
-        <v>15881</v>
+        <v>19021</v>
       </c>
       <c r="N18" t="n">
-        <v>37775</v>
+        <v>43268</v>
       </c>
     </row>
     <row r="19">
@@ -1283,13 +1283,13 @@
         <v>55231</v>
       </c>
       <c r="L19" t="n">
-        <v>33416</v>
+        <v>38194</v>
       </c>
       <c r="M19" t="n">
-        <v>9335</v>
+        <v>11043</v>
       </c>
       <c r="N19" t="n">
-        <v>24081</v>
+        <v>27151</v>
       </c>
     </row>
     <row r="20">
@@ -1327,13 +1327,13 @@
         <v>58737</v>
       </c>
       <c r="L20" t="n">
-        <v>28248</v>
+        <v>34355</v>
       </c>
       <c r="M20" t="n">
-        <v>7554</v>
+        <v>9159</v>
       </c>
       <c r="N20" t="n">
-        <v>20694</v>
+        <v>25196</v>
       </c>
     </row>
     <row r="21">
@@ -1371,13 +1371,13 @@
         <v>24382</v>
       </c>
       <c r="L21" t="n">
-        <v>10815</v>
+        <v>13581</v>
       </c>
       <c r="M21" t="n">
-        <v>2949</v>
+        <v>3662</v>
       </c>
       <c r="N21" t="n">
-        <v>7866</v>
+        <v>9919</v>
       </c>
     </row>
     <row r="22">
@@ -1415,13 +1415,13 @@
         <v>152229</v>
       </c>
       <c r="L22" t="n">
-        <v>58868</v>
+        <v>68055</v>
       </c>
       <c r="M22" t="n">
-        <v>15702</v>
+        <v>18661</v>
       </c>
       <c r="N22" t="n">
-        <v>43166</v>
+        <v>49394</v>
       </c>
     </row>
     <row r="23">
@@ -1459,13 +1459,13 @@
         <v>40867</v>
       </c>
       <c r="L23" t="n">
-        <v>21833</v>
+        <v>24978</v>
       </c>
       <c r="M23" t="n">
-        <v>5102</v>
+        <v>5975</v>
       </c>
       <c r="N23" t="n">
-        <v>16731</v>
+        <v>19003</v>
       </c>
     </row>
     <row r="24">
@@ -1503,13 +1503,13 @@
         <v>88798</v>
       </c>
       <c r="L24" t="n">
-        <v>70489</v>
+        <v>83588</v>
       </c>
       <c r="M24" t="n">
-        <v>15718</v>
+        <v>19255</v>
       </c>
       <c r="N24" t="n">
-        <v>54771</v>
+        <v>64333</v>
       </c>
     </row>
     <row r="25">
@@ -1547,13 +1547,13 @@
         <v>86600</v>
       </c>
       <c r="L25" t="n">
-        <v>47096</v>
+        <v>55707</v>
       </c>
       <c r="M25" t="n">
-        <v>16203</v>
+        <v>19424</v>
       </c>
       <c r="N25" t="n">
-        <v>30893</v>
+        <v>36283</v>
       </c>
     </row>
     <row r="26">
@@ -1591,13 +1591,13 @@
         <v>95605</v>
       </c>
       <c r="L26" t="n">
-        <v>70975</v>
+        <v>84295</v>
       </c>
       <c r="M26" t="n">
-        <v>23108</v>
+        <v>28200</v>
       </c>
       <c r="N26" t="n">
-        <v>47867</v>
+        <v>56095</v>
       </c>
     </row>
     <row r="27">
@@ -1635,13 +1635,13 @@
         <v>35197</v>
       </c>
       <c r="L27" t="n">
-        <v>25830</v>
+        <v>30172</v>
       </c>
       <c r="M27" t="n">
-        <v>7358</v>
+        <v>8773</v>
       </c>
       <c r="N27" t="n">
-        <v>18472</v>
+        <v>21399</v>
       </c>
     </row>
     <row r="28">
@@ -1679,13 +1679,13 @@
         <v>52800</v>
       </c>
       <c r="L28" t="n">
-        <v>38075</v>
+        <v>43714</v>
       </c>
       <c r="M28" t="n">
-        <v>6206</v>
+        <v>7382</v>
       </c>
       <c r="N28" t="n">
-        <v>31869</v>
+        <v>36332</v>
       </c>
     </row>
     <row r="29">
@@ -1723,13 +1723,13 @@
         <v>34093</v>
       </c>
       <c r="L29" t="n">
-        <v>23465</v>
+        <v>27541</v>
       </c>
       <c r="M29" t="n">
-        <v>3946</v>
+        <v>4767</v>
       </c>
       <c r="N29" t="n">
-        <v>19519</v>
+        <v>22774</v>
       </c>
     </row>
     <row r="30">
@@ -1767,13 +1767,13 @@
         <v>59519</v>
       </c>
       <c r="L30" t="n">
-        <v>23391</v>
+        <v>27208</v>
       </c>
       <c r="M30" t="n">
-        <v>4215</v>
+        <v>5150</v>
       </c>
       <c r="N30" t="n">
-        <v>19176</v>
+        <v>22058</v>
       </c>
     </row>
     <row r="31">
@@ -1811,13 +1811,13 @@
         <v>111215</v>
       </c>
       <c r="L31" t="n">
-        <v>49528</v>
+        <v>59196</v>
       </c>
       <c r="M31" t="n">
-        <v>11623</v>
+        <v>14310</v>
       </c>
       <c r="N31" t="n">
-        <v>37905</v>
+        <v>44886</v>
       </c>
     </row>
     <row r="32">
@@ -1855,13 +1855,13 @@
         <v>135620</v>
       </c>
       <c r="L32" t="n">
-        <v>52818</v>
+        <v>63031</v>
       </c>
       <c r="M32" t="n">
-        <v>13326</v>
+        <v>15993</v>
       </c>
       <c r="N32" t="n">
-        <v>39492</v>
+        <v>47038</v>
       </c>
     </row>
     <row r="33">
@@ -1899,13 +1899,13 @@
         <v>46108</v>
       </c>
       <c r="L33" t="n">
-        <v>36461</v>
+        <v>42474</v>
       </c>
       <c r="M33" t="n">
-        <v>12197</v>
+        <v>14680</v>
       </c>
       <c r="N33" t="n">
-        <v>24264</v>
+        <v>27794</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>74035</v>
       </c>
       <c r="L34" t="n">
-        <v>37860</v>
+        <v>43128</v>
       </c>
       <c r="M34" t="n">
-        <v>7928</v>
+        <v>9468</v>
       </c>
       <c r="N34" t="n">
-        <v>29932</v>
+        <v>33660</v>
       </c>
     </row>
     <row r="35">
@@ -1987,13 +1987,13 @@
         <v>134411</v>
       </c>
       <c r="L35" t="n">
-        <v>50347</v>
+        <v>60881</v>
       </c>
       <c r="M35" t="n">
-        <v>10212</v>
+        <v>12567</v>
       </c>
       <c r="N35" t="n">
-        <v>40135</v>
+        <v>48314</v>
       </c>
     </row>
     <row r="36">
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>39307</v>
+        <v>46859</v>
       </c>
       <c r="M36" t="n">
-        <v>7188</v>
+        <v>9031</v>
       </c>
       <c r="N36" t="n">
-        <v>32119</v>
+        <v>37828</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>62713</v>
+        <v>73311</v>
       </c>
       <c r="M37" t="n">
-        <v>21119</v>
+        <v>25918</v>
       </c>
       <c r="N37" t="n">
-        <v>41594</v>
+        <v>47393</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>13683</v>
+        <v>15737</v>
       </c>
       <c r="M38" t="n">
-        <v>2257</v>
+        <v>2691</v>
       </c>
       <c r="N38" t="n">
-        <v>11426</v>
+        <v>13046</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>14649</v>
+        <v>17076</v>
       </c>
       <c r="M39" t="n">
-        <v>3084</v>
+        <v>3720</v>
       </c>
       <c r="N39" t="n">
-        <v>11565</v>
+        <v>13356</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>41630</v>
+        <v>49203</v>
       </c>
       <c r="M40" t="n">
-        <v>7535</v>
+        <v>9186</v>
       </c>
       <c r="N40" t="n">
-        <v>34095</v>
+        <v>40017</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>6291</v>
+        <v>7432</v>
       </c>
       <c r="M41" t="n">
-        <v>894</v>
+        <v>1118</v>
       </c>
       <c r="N41" t="n">
-        <v>5397</v>
+        <v>6314</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>44589</v>
+        <v>51174</v>
       </c>
       <c r="M42" t="n">
-        <v>8771</v>
+        <v>10470</v>
       </c>
       <c r="N42" t="n">
-        <v>35818</v>
+        <v>40704</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>30827</v>
+        <v>36083</v>
       </c>
       <c r="M43" t="n">
-        <v>7265</v>
+        <v>8674</v>
       </c>
       <c r="N43" t="n">
-        <v>23562</v>
+        <v>27409</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>57630</v>
+        <v>66958</v>
       </c>
       <c r="M44" t="n">
-        <v>15642</v>
+        <v>18960</v>
       </c>
       <c r="N44" t="n">
-        <v>41988</v>
+        <v>47998</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>39346</v>
+        <v>46900</v>
       </c>
       <c r="M45" t="n">
-        <v>8167</v>
+        <v>10157</v>
       </c>
       <c r="N45" t="n">
-        <v>31179</v>
+        <v>36743</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>52371</v>
+        <v>61381</v>
       </c>
       <c r="M46" t="n">
-        <v>8403</v>
+        <v>10382</v>
       </c>
       <c r="N46" t="n">
-        <v>43968</v>
+        <v>50999</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>99207</v>
+        <v>118938</v>
       </c>
       <c r="M47" t="n">
-        <v>42350</v>
+        <v>51202</v>
       </c>
       <c r="N47" t="n">
-        <v>56857</v>
+        <v>67736</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>101644</v>
+        <v>119611</v>
       </c>
       <c r="M48" t="n">
-        <v>41171</v>
+        <v>50427</v>
       </c>
       <c r="N48" t="n">
-        <v>60473</v>
+        <v>69184</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>38308</v>
+        <v>45355</v>
       </c>
       <c r="M49" t="n">
-        <v>11280</v>
+        <v>13961</v>
       </c>
       <c r="N49" t="n">
-        <v>27028</v>
+        <v>31394</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>34088</v>
+        <v>39063</v>
       </c>
       <c r="M50" t="n">
-        <v>4266</v>
+        <v>5082</v>
       </c>
       <c r="N50" t="n">
-        <v>29822</v>
+        <v>33981</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>15822</v>
+        <v>18732</v>
       </c>
       <c r="M51" t="n">
-        <v>3532</v>
+        <v>4352</v>
       </c>
       <c r="N51" t="n">
-        <v>12290</v>
+        <v>14380</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>39827</v>
+        <v>46325</v>
       </c>
       <c r="M52" t="n">
-        <v>9572</v>
+        <v>11868</v>
       </c>
       <c r="N52" t="n">
-        <v>30255</v>
+        <v>34457</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>29069</v>
+        <v>33219</v>
       </c>
       <c r="M53" t="n">
-        <v>7115</v>
+        <v>8542</v>
       </c>
       <c r="N53" t="n">
-        <v>21954</v>
+        <v>24677</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>24610</v>
+        <v>29857</v>
       </c>
       <c r="M54" t="n">
-        <v>6247</v>
+        <v>7624</v>
       </c>
       <c r="N54" t="n">
-        <v>18363</v>
+        <v>22233</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>8997</v>
+        <v>11289</v>
       </c>
       <c r="M55" t="n">
-        <v>2320</v>
+        <v>2921</v>
       </c>
       <c r="N55" t="n">
-        <v>6677</v>
+        <v>8368</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>51552</v>
+        <v>59545</v>
       </c>
       <c r="M56" t="n">
-        <v>12265</v>
+        <v>14776</v>
       </c>
       <c r="N56" t="n">
-        <v>39287</v>
+        <v>44769</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>19325</v>
+        <v>22040</v>
       </c>
       <c r="M57" t="n">
-        <v>4256</v>
+        <v>5000</v>
       </c>
       <c r="N57" t="n">
-        <v>15069</v>
+        <v>17040</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>59970</v>
+        <v>71031</v>
       </c>
       <c r="M58" t="n">
-        <v>11281</v>
+        <v>14117</v>
       </c>
       <c r="N58" t="n">
-        <v>48689</v>
+        <v>56914</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>33530</v>
+        <v>39971</v>
       </c>
       <c r="M59" t="n">
-        <v>9228</v>
+        <v>11550</v>
       </c>
       <c r="N59" t="n">
-        <v>24302</v>
+        <v>28421</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>56818</v>
+        <v>67566</v>
       </c>
       <c r="M60" t="n">
-        <v>16179</v>
+        <v>20179</v>
       </c>
       <c r="N60" t="n">
-        <v>40639</v>
+        <v>47387</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>19462</v>
+        <v>22848</v>
       </c>
       <c r="M61" t="n">
-        <v>4769</v>
+        <v>5805</v>
       </c>
       <c r="N61" t="n">
-        <v>14693</v>
+        <v>17043</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>34589</v>
+        <v>39624</v>
       </c>
       <c r="M62" t="n">
-        <v>4821</v>
+        <v>5811</v>
       </c>
       <c r="N62" t="n">
-        <v>29768</v>
+        <v>33813</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>19635</v>
+        <v>22912</v>
       </c>
       <c r="M63" t="n">
-        <v>2720</v>
+        <v>3370</v>
       </c>
       <c r="N63" t="n">
-        <v>16915</v>
+        <v>19542</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>20549</v>
+        <v>23864</v>
       </c>
       <c r="M64" t="n">
-        <v>3479</v>
+        <v>4289</v>
       </c>
       <c r="N64" t="n">
-        <v>17070</v>
+        <v>19575</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>39845</v>
+        <v>47680</v>
       </c>
       <c r="M65" t="n">
-        <v>7766</v>
+        <v>9851</v>
       </c>
       <c r="N65" t="n">
-        <v>32079</v>
+        <v>37829</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>40947</v>
+        <v>49252</v>
       </c>
       <c r="M66" t="n">
-        <v>8182</v>
+        <v>10178</v>
       </c>
       <c r="N66" t="n">
-        <v>32765</v>
+        <v>39074</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>31014</v>
+        <v>36131</v>
       </c>
       <c r="M67" t="n">
-        <v>9149</v>
+        <v>11203</v>
       </c>
       <c r="N67" t="n">
-        <v>21865</v>
+        <v>24928</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>33485</v>
+        <v>38022</v>
       </c>
       <c r="M68" t="n">
-        <v>6719</v>
+        <v>8044</v>
       </c>
       <c r="N68" t="n">
-        <v>26766</v>
+        <v>29978</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>42102</v>
+        <v>51011</v>
       </c>
       <c r="M69" t="n">
-        <v>6797</v>
+        <v>8593</v>
       </c>
       <c r="N69" t="n">
-        <v>35305</v>
+        <v>42418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboard data for 2026-04-28
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -535,13 +535,13 @@
         <v>150469</v>
       </c>
       <c r="L2" t="n">
-        <v>58428</v>
+        <v>67491</v>
       </c>
       <c r="M2" t="n">
-        <v>13110</v>
+        <v>15230</v>
       </c>
       <c r="N2" t="n">
-        <v>45318</v>
+        <v>52261</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>81428</v>
       </c>
       <c r="L3" t="n">
-        <v>95067</v>
+        <v>108267</v>
       </c>
       <c r="M3" t="n">
-        <v>38520</v>
+        <v>43897</v>
       </c>
       <c r="N3" t="n">
-        <v>56547</v>
+        <v>64370</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +623,13 @@
         <v>18713</v>
       </c>
       <c r="L4" t="n">
-        <v>16985</v>
+        <v>19849</v>
       </c>
       <c r="M4" t="n">
-        <v>3063</v>
+        <v>3583</v>
       </c>
       <c r="N4" t="n">
-        <v>13922</v>
+        <v>16266</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         <v>42408</v>
       </c>
       <c r="L5" t="n">
-        <v>21521</v>
+        <v>24840</v>
       </c>
       <c r="M5" t="n">
-        <v>5893</v>
+        <v>6742</v>
       </c>
       <c r="N5" t="n">
-        <v>15628</v>
+        <v>18098</v>
       </c>
     </row>
     <row r="6">
@@ -711,13 +711,13 @@
         <v>117439</v>
       </c>
       <c r="L6" t="n">
-        <v>61859</v>
+        <v>71428</v>
       </c>
       <c r="M6" t="n">
-        <v>14733</v>
+        <v>16777</v>
       </c>
       <c r="N6" t="n">
-        <v>47126</v>
+        <v>54651</v>
       </c>
     </row>
     <row r="7">
@@ -755,13 +755,13 @@
         <v>19076</v>
       </c>
       <c r="L7" t="n">
-        <v>8872</v>
+        <v>9944</v>
       </c>
       <c r="M7" t="n">
-        <v>1444</v>
+        <v>1649</v>
       </c>
       <c r="N7" t="n">
-        <v>7428</v>
+        <v>8295</v>
       </c>
     </row>
     <row r="8">
@@ -799,13 +799,13 @@
         <v>83014</v>
       </c>
       <c r="L8" t="n">
-        <v>57942</v>
+        <v>66979</v>
       </c>
       <c r="M8" t="n">
-        <v>12877</v>
+        <v>14900</v>
       </c>
       <c r="N8" t="n">
-        <v>45065</v>
+        <v>52079</v>
       </c>
     </row>
     <row r="9">
@@ -843,13 +843,13 @@
         <v>65107</v>
       </c>
       <c r="L9" t="n">
-        <v>43797</v>
+        <v>50146</v>
       </c>
       <c r="M9" t="n">
-        <v>13283</v>
+        <v>15378</v>
       </c>
       <c r="N9" t="n">
-        <v>30514</v>
+        <v>34768</v>
       </c>
     </row>
     <row r="10">
@@ -887,13 +887,13 @@
         <v>151451</v>
       </c>
       <c r="L10" t="n">
-        <v>81959</v>
+        <v>93311</v>
       </c>
       <c r="M10" t="n">
-        <v>27452</v>
+        <v>31174</v>
       </c>
       <c r="N10" t="n">
-        <v>54507</v>
+        <v>62137</v>
       </c>
     </row>
     <row r="11">
@@ -931,13 +931,13 @@
         <v>127517</v>
       </c>
       <c r="L11" t="n">
-        <v>57074</v>
+        <v>67238</v>
       </c>
       <c r="M11" t="n">
-        <v>14202</v>
+        <v>16442</v>
       </c>
       <c r="N11" t="n">
-        <v>42872</v>
+        <v>50796</v>
       </c>
     </row>
     <row r="12">
@@ -975,13 +975,13 @@
         <v>122266</v>
       </c>
       <c r="L12" t="n">
-        <v>69826</v>
+        <v>80754</v>
       </c>
       <c r="M12" t="n">
-        <v>13246</v>
+        <v>15507</v>
       </c>
       <c r="N12" t="n">
-        <v>56580</v>
+        <v>65247</v>
       </c>
     </row>
     <row r="13">
@@ -1019,13 +1019,13 @@
         <v>399425</v>
       </c>
       <c r="L13" t="n">
-        <v>183303</v>
+        <v>215088</v>
       </c>
       <c r="M13" t="n">
-        <v>93836</v>
+        <v>107015</v>
       </c>
       <c r="N13" t="n">
-        <v>89467</v>
+        <v>108073</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         <v>274795</v>
       </c>
       <c r="L14" t="n">
-        <v>204790</v>
+        <v>240276</v>
       </c>
       <c r="M14" t="n">
-        <v>100981</v>
+        <v>115973</v>
       </c>
       <c r="N14" t="n">
-        <v>103809</v>
+        <v>124303</v>
       </c>
     </row>
     <row r="15">
@@ -1107,13 +1107,13 @@
         <v>80530</v>
       </c>
       <c r="L15" t="n">
-        <v>65401</v>
+        <v>75718</v>
       </c>
       <c r="M15" t="n">
-        <v>23582</v>
+        <v>26878</v>
       </c>
       <c r="N15" t="n">
-        <v>41819</v>
+        <v>48840</v>
       </c>
     </row>
     <row r="16">
@@ -1151,13 +1151,13 @@
         <v>15975</v>
       </c>
       <c r="L16" t="n">
-        <v>45918</v>
+        <v>51316</v>
       </c>
       <c r="M16" t="n">
-        <v>7006</v>
+        <v>7910</v>
       </c>
       <c r="N16" t="n">
-        <v>38912</v>
+        <v>43406</v>
       </c>
     </row>
     <row r="17">
@@ -1195,13 +1195,13 @@
         <v>26564</v>
       </c>
       <c r="L17" t="n">
-        <v>23028</v>
+        <v>26726</v>
       </c>
       <c r="M17" t="n">
-        <v>6581</v>
+        <v>7541</v>
       </c>
       <c r="N17" t="n">
-        <v>16447</v>
+        <v>19185</v>
       </c>
     </row>
     <row r="18">
@@ -1239,13 +1239,13 @@
         <v>66764</v>
       </c>
       <c r="L18" t="n">
-        <v>62289</v>
+        <v>70870</v>
       </c>
       <c r="M18" t="n">
-        <v>19021</v>
+        <v>21736</v>
       </c>
       <c r="N18" t="n">
-        <v>43268</v>
+        <v>49134</v>
       </c>
     </row>
     <row r="19">
@@ -1283,13 +1283,13 @@
         <v>55231</v>
       </c>
       <c r="L19" t="n">
-        <v>38194</v>
+        <v>43592</v>
       </c>
       <c r="M19" t="n">
-        <v>11043</v>
+        <v>12626</v>
       </c>
       <c r="N19" t="n">
-        <v>27151</v>
+        <v>30966</v>
       </c>
     </row>
     <row r="20">
@@ -1327,13 +1327,13 @@
         <v>58737</v>
       </c>
       <c r="L20" t="n">
-        <v>34355</v>
+        <v>40208</v>
       </c>
       <c r="M20" t="n">
-        <v>9159</v>
+        <v>10492</v>
       </c>
       <c r="N20" t="n">
-        <v>25196</v>
+        <v>29716</v>
       </c>
     </row>
     <row r="21">
@@ -1371,13 +1371,13 @@
         <v>24382</v>
       </c>
       <c r="L21" t="n">
-        <v>13581</v>
+        <v>15632</v>
       </c>
       <c r="M21" t="n">
-        <v>3662</v>
+        <v>4284</v>
       </c>
       <c r="N21" t="n">
-        <v>9919</v>
+        <v>11348</v>
       </c>
     </row>
     <row r="22">
@@ -1415,13 +1415,13 @@
         <v>152229</v>
       </c>
       <c r="L22" t="n">
-        <v>68055</v>
+        <v>79087</v>
       </c>
       <c r="M22" t="n">
-        <v>18661</v>
+        <v>21671</v>
       </c>
       <c r="N22" t="n">
-        <v>49394</v>
+        <v>57416</v>
       </c>
     </row>
     <row r="23">
@@ -1459,13 +1459,13 @@
         <v>40867</v>
       </c>
       <c r="L23" t="n">
-        <v>24978</v>
+        <v>28778</v>
       </c>
       <c r="M23" t="n">
-        <v>5975</v>
+        <v>6804</v>
       </c>
       <c r="N23" t="n">
-        <v>19003</v>
+        <v>21974</v>
       </c>
     </row>
     <row r="24">
@@ -1503,13 +1503,13 @@
         <v>88798</v>
       </c>
       <c r="L24" t="n">
-        <v>83588</v>
+        <v>94007</v>
       </c>
       <c r="M24" t="n">
-        <v>19255</v>
+        <v>22133</v>
       </c>
       <c r="N24" t="n">
-        <v>64333</v>
+        <v>71874</v>
       </c>
     </row>
     <row r="25">
@@ -1547,13 +1547,13 @@
         <v>86600</v>
       </c>
       <c r="L25" t="n">
-        <v>55707</v>
+        <v>64398</v>
       </c>
       <c r="M25" t="n">
-        <v>19424</v>
+        <v>22189</v>
       </c>
       <c r="N25" t="n">
-        <v>36283</v>
+        <v>42209</v>
       </c>
     </row>
     <row r="26">
@@ -1591,13 +1591,13 @@
         <v>95605</v>
       </c>
       <c r="L26" t="n">
-        <v>84295</v>
+        <v>97934</v>
       </c>
       <c r="M26" t="n">
-        <v>28200</v>
+        <v>32443</v>
       </c>
       <c r="N26" t="n">
-        <v>56095</v>
+        <v>65491</v>
       </c>
     </row>
     <row r="27">
@@ -1635,13 +1635,13 @@
         <v>35197</v>
       </c>
       <c r="L27" t="n">
-        <v>30172</v>
+        <v>35008</v>
       </c>
       <c r="M27" t="n">
-        <v>8773</v>
+        <v>10112</v>
       </c>
       <c r="N27" t="n">
-        <v>21399</v>
+        <v>24896</v>
       </c>
     </row>
     <row r="28">
@@ -1679,13 +1679,13 @@
         <v>52800</v>
       </c>
       <c r="L28" t="n">
-        <v>43714</v>
+        <v>50053</v>
       </c>
       <c r="M28" t="n">
-        <v>7382</v>
+        <v>8481</v>
       </c>
       <c r="N28" t="n">
-        <v>36332</v>
+        <v>41572</v>
       </c>
     </row>
     <row r="29">
@@ -1723,13 +1723,13 @@
         <v>34093</v>
       </c>
       <c r="L29" t="n">
-        <v>27541</v>
+        <v>32058</v>
       </c>
       <c r="M29" t="n">
-        <v>4767</v>
+        <v>5450</v>
       </c>
       <c r="N29" t="n">
-        <v>22774</v>
+        <v>26608</v>
       </c>
     </row>
     <row r="30">
@@ -1767,13 +1767,13 @@
         <v>59519</v>
       </c>
       <c r="L30" t="n">
-        <v>27208</v>
+        <v>30744</v>
       </c>
       <c r="M30" t="n">
-        <v>5150</v>
+        <v>5934</v>
       </c>
       <c r="N30" t="n">
-        <v>22058</v>
+        <v>24810</v>
       </c>
     </row>
     <row r="31">
@@ -1811,13 +1811,13 @@
         <v>111215</v>
       </c>
       <c r="L31" t="n">
-        <v>59196</v>
+        <v>67843</v>
       </c>
       <c r="M31" t="n">
-        <v>14310</v>
+        <v>16543</v>
       </c>
       <c r="N31" t="n">
-        <v>44886</v>
+        <v>51300</v>
       </c>
     </row>
     <row r="32">
@@ -1855,13 +1855,13 @@
         <v>135620</v>
       </c>
       <c r="L32" t="n">
-        <v>63031</v>
+        <v>73512</v>
       </c>
       <c r="M32" t="n">
-        <v>15993</v>
+        <v>18187</v>
       </c>
       <c r="N32" t="n">
-        <v>47038</v>
+        <v>55325</v>
       </c>
     </row>
     <row r="33">
@@ -1899,13 +1899,13 @@
         <v>46108</v>
       </c>
       <c r="L33" t="n">
-        <v>42474</v>
+        <v>48923</v>
       </c>
       <c r="M33" t="n">
-        <v>14680</v>
+        <v>16731</v>
       </c>
       <c r="N33" t="n">
-        <v>27794</v>
+        <v>32192</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>74035</v>
       </c>
       <c r="L34" t="n">
-        <v>43128</v>
+        <v>48207</v>
       </c>
       <c r="M34" t="n">
-        <v>9468</v>
+        <v>10666</v>
       </c>
       <c r="N34" t="n">
-        <v>33660</v>
+        <v>37541</v>
       </c>
     </row>
     <row r="35">
@@ -1987,13 +1987,13 @@
         <v>134411</v>
       </c>
       <c r="L35" t="n">
-        <v>60881</v>
+        <v>72687</v>
       </c>
       <c r="M35" t="n">
-        <v>12567</v>
+        <v>14782</v>
       </c>
       <c r="N35" t="n">
-        <v>48314</v>
+        <v>57905</v>
       </c>
     </row>
     <row r="36">
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>46859</v>
+        <v>51905</v>
       </c>
       <c r="M36" t="n">
-        <v>9031</v>
+        <v>10130</v>
       </c>
       <c r="N36" t="n">
-        <v>37828</v>
+        <v>41775</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>73311</v>
+        <v>81833</v>
       </c>
       <c r="M37" t="n">
-        <v>25918</v>
+        <v>29137</v>
       </c>
       <c r="N37" t="n">
-        <v>47393</v>
+        <v>52696</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>15737</v>
+        <v>17592</v>
       </c>
       <c r="M38" t="n">
-        <v>2691</v>
+        <v>3022</v>
       </c>
       <c r="N38" t="n">
-        <v>13046</v>
+        <v>14570</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>17076</v>
+        <v>18530</v>
       </c>
       <c r="M39" t="n">
-        <v>3720</v>
+        <v>4003</v>
       </c>
       <c r="N39" t="n">
-        <v>13356</v>
+        <v>14527</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>49203</v>
+        <v>54258</v>
       </c>
       <c r="M40" t="n">
-        <v>9186</v>
+        <v>10071</v>
       </c>
       <c r="N40" t="n">
-        <v>40017</v>
+        <v>44187</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>7432</v>
+        <v>8007</v>
       </c>
       <c r="M41" t="n">
-        <v>1118</v>
+        <v>1222</v>
       </c>
       <c r="N41" t="n">
-        <v>6314</v>
+        <v>6785</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>51174</v>
+        <v>57099</v>
       </c>
       <c r="M42" t="n">
-        <v>10470</v>
+        <v>11749</v>
       </c>
       <c r="N42" t="n">
-        <v>40704</v>
+        <v>45350</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>36083</v>
+        <v>39789</v>
       </c>
       <c r="M43" t="n">
-        <v>8674</v>
+        <v>9639</v>
       </c>
       <c r="N43" t="n">
-        <v>27409</v>
+        <v>30150</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>66958</v>
+        <v>74153</v>
       </c>
       <c r="M44" t="n">
-        <v>18960</v>
+        <v>21046</v>
       </c>
       <c r="N44" t="n">
-        <v>47998</v>
+        <v>53107</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>46900</v>
+        <v>53145</v>
       </c>
       <c r="M45" t="n">
-        <v>10157</v>
+        <v>11447</v>
       </c>
       <c r="N45" t="n">
-        <v>36743</v>
+        <v>41698</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>61381</v>
+        <v>68482</v>
       </c>
       <c r="M46" t="n">
-        <v>10382</v>
+        <v>11829</v>
       </c>
       <c r="N46" t="n">
-        <v>50999</v>
+        <v>56653</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>118938</v>
+        <v>135411</v>
       </c>
       <c r="M47" t="n">
-        <v>51202</v>
+        <v>57467</v>
       </c>
       <c r="N47" t="n">
-        <v>67736</v>
+        <v>77944</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>119611</v>
+        <v>135702</v>
       </c>
       <c r="M48" t="n">
-        <v>50427</v>
+        <v>56765</v>
       </c>
       <c r="N48" t="n">
-        <v>69184</v>
+        <v>78937</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>45355</v>
+        <v>50794</v>
       </c>
       <c r="M49" t="n">
-        <v>13961</v>
+        <v>15564</v>
       </c>
       <c r="N49" t="n">
-        <v>31394</v>
+        <v>35230</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>39063</v>
+        <v>42332</v>
       </c>
       <c r="M50" t="n">
-        <v>5082</v>
+        <v>5600</v>
       </c>
       <c r="N50" t="n">
-        <v>33981</v>
+        <v>36732</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>18732</v>
+        <v>21152</v>
       </c>
       <c r="M51" t="n">
-        <v>4352</v>
+        <v>4869</v>
       </c>
       <c r="N51" t="n">
-        <v>14380</v>
+        <v>16283</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>46325</v>
+        <v>50713</v>
       </c>
       <c r="M52" t="n">
-        <v>11868</v>
+        <v>13228</v>
       </c>
       <c r="N52" t="n">
-        <v>34457</v>
+        <v>37485</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>33219</v>
+        <v>37039</v>
       </c>
       <c r="M53" t="n">
-        <v>8542</v>
+        <v>9553</v>
       </c>
       <c r="N53" t="n">
-        <v>24677</v>
+        <v>27486</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>29857</v>
+        <v>33217</v>
       </c>
       <c r="M54" t="n">
-        <v>7624</v>
+        <v>8390</v>
       </c>
       <c r="N54" t="n">
-        <v>22233</v>
+        <v>24827</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>11289</v>
+        <v>12106</v>
       </c>
       <c r="M55" t="n">
-        <v>2921</v>
+        <v>3159</v>
       </c>
       <c r="N55" t="n">
-        <v>8368</v>
+        <v>8947</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>59545</v>
+        <v>67007</v>
       </c>
       <c r="M56" t="n">
-        <v>14776</v>
+        <v>16695</v>
       </c>
       <c r="N56" t="n">
-        <v>44769</v>
+        <v>50312</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>22040</v>
+        <v>24060</v>
       </c>
       <c r="M57" t="n">
-        <v>5000</v>
+        <v>5453</v>
       </c>
       <c r="N57" t="n">
-        <v>17040</v>
+        <v>18607</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>71031</v>
+        <v>76964</v>
       </c>
       <c r="M58" t="n">
-        <v>14117</v>
+        <v>15674</v>
       </c>
       <c r="N58" t="n">
-        <v>56914</v>
+        <v>61290</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>39971</v>
+        <v>44550</v>
       </c>
       <c r="M59" t="n">
-        <v>11550</v>
+        <v>12846</v>
       </c>
       <c r="N59" t="n">
-        <v>28421</v>
+        <v>31704</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>67566</v>
+        <v>75713</v>
       </c>
       <c r="M60" t="n">
-        <v>20179</v>
+        <v>22551</v>
       </c>
       <c r="N60" t="n">
-        <v>47387</v>
+        <v>53162</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>22848</v>
+        <v>25353</v>
       </c>
       <c r="M61" t="n">
-        <v>5805</v>
+        <v>6442</v>
       </c>
       <c r="N61" t="n">
-        <v>17043</v>
+        <v>18911</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>39624</v>
+        <v>44225</v>
       </c>
       <c r="M62" t="n">
-        <v>5811</v>
+        <v>6509</v>
       </c>
       <c r="N62" t="n">
-        <v>33813</v>
+        <v>37716</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>22912</v>
+        <v>25224</v>
       </c>
       <c r="M63" t="n">
-        <v>3370</v>
+        <v>3742</v>
       </c>
       <c r="N63" t="n">
-        <v>19542</v>
+        <v>21482</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>23864</v>
+        <v>25937</v>
       </c>
       <c r="M64" t="n">
-        <v>4289</v>
+        <v>4744</v>
       </c>
       <c r="N64" t="n">
-        <v>19575</v>
+        <v>21193</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>47680</v>
+        <v>52376</v>
       </c>
       <c r="M65" t="n">
-        <v>9851</v>
+        <v>10999</v>
       </c>
       <c r="N65" t="n">
-        <v>37829</v>
+        <v>41377</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>49252</v>
+        <v>55387</v>
       </c>
       <c r="M66" t="n">
-        <v>10178</v>
+        <v>11296</v>
       </c>
       <c r="N66" t="n">
-        <v>39074</v>
+        <v>44091</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>36131</v>
+        <v>40684</v>
       </c>
       <c r="M67" t="n">
-        <v>11203</v>
+        <v>12525</v>
       </c>
       <c r="N67" t="n">
-        <v>24928</v>
+        <v>28159</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>38022</v>
+        <v>40993</v>
       </c>
       <c r="M68" t="n">
-        <v>8044</v>
+        <v>8713</v>
       </c>
       <c r="N68" t="n">
-        <v>29978</v>
+        <v>32280</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>51011</v>
+        <v>58355</v>
       </c>
       <c r="M69" t="n">
-        <v>8593</v>
+        <v>9756</v>
       </c>
       <c r="N69" t="n">
-        <v>42418</v>
+        <v>48599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data for 20260428: add VBI data, regenerate reports
</commit_message>
<xml_diff>
--- a/f_total_cap_nhat.xlsx
+++ b/f_total_cap_nhat.xlsx
@@ -2031,13 +2031,13 @@
         <v>93875</v>
       </c>
       <c r="L36" t="n">
-        <v>51905</v>
+        <v>54068</v>
       </c>
       <c r="M36" t="n">
-        <v>10130</v>
+        <v>10539</v>
       </c>
       <c r="N36" t="n">
-        <v>41775</v>
+        <v>43529</v>
       </c>
     </row>
     <row r="37">
@@ -2075,13 +2075,13 @@
         <v>65690</v>
       </c>
       <c r="L37" t="n">
-        <v>81833</v>
+        <v>83403</v>
       </c>
       <c r="M37" t="n">
-        <v>29137</v>
+        <v>29599</v>
       </c>
       <c r="N37" t="n">
-        <v>52696</v>
+        <v>53804</v>
       </c>
     </row>
     <row r="38">
@@ -2119,13 +2119,13 @@
         <v>7829</v>
       </c>
       <c r="L38" t="n">
-        <v>17592</v>
+        <v>18338</v>
       </c>
       <c r="M38" t="n">
-        <v>3022</v>
+        <v>3149</v>
       </c>
       <c r="N38" t="n">
-        <v>14570</v>
+        <v>15189</v>
       </c>
     </row>
     <row r="39">
@@ -2163,13 +2163,13 @@
         <v>26289</v>
       </c>
       <c r="L39" t="n">
-        <v>18530</v>
+        <v>19747</v>
       </c>
       <c r="M39" t="n">
-        <v>4003</v>
+        <v>4294</v>
       </c>
       <c r="N39" t="n">
-        <v>14527</v>
+        <v>15453</v>
       </c>
     </row>
     <row r="40">
@@ -2207,13 +2207,13 @@
         <v>74072</v>
       </c>
       <c r="L40" t="n">
-        <v>54258</v>
+        <v>56732</v>
       </c>
       <c r="M40" t="n">
-        <v>10071</v>
+        <v>10482</v>
       </c>
       <c r="N40" t="n">
-        <v>44187</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="41">
@@ -2251,13 +2251,13 @@
         <v>11564</v>
       </c>
       <c r="L41" t="n">
-        <v>8007</v>
+        <v>8335</v>
       </c>
       <c r="M41" t="n">
-        <v>1222</v>
+        <v>1275</v>
       </c>
       <c r="N41" t="n">
-        <v>6785</v>
+        <v>7060</v>
       </c>
     </row>
     <row r="42">
@@ -2295,13 +2295,13 @@
         <v>41594</v>
       </c>
       <c r="L42" t="n">
-        <v>57099</v>
+        <v>59151</v>
       </c>
       <c r="M42" t="n">
-        <v>11749</v>
+        <v>12148</v>
       </c>
       <c r="N42" t="n">
-        <v>45350</v>
+        <v>47003</v>
       </c>
     </row>
     <row r="43">
@@ -2339,13 +2339,13 @@
         <v>39097</v>
       </c>
       <c r="L43" t="n">
-        <v>39789</v>
+        <v>41035</v>
       </c>
       <c r="M43" t="n">
-        <v>9639</v>
+        <v>9938</v>
       </c>
       <c r="N43" t="n">
-        <v>30150</v>
+        <v>31097</v>
       </c>
     </row>
     <row r="44">
@@ -2383,13 +2383,13 @@
         <v>90813</v>
       </c>
       <c r="L44" t="n">
-        <v>74153</v>
+        <v>75972</v>
       </c>
       <c r="M44" t="n">
-        <v>21046</v>
+        <v>21474</v>
       </c>
       <c r="N44" t="n">
-        <v>53107</v>
+        <v>54498</v>
       </c>
     </row>
     <row r="45">
@@ -2427,13 +2427,13 @@
         <v>74362</v>
       </c>
       <c r="L45" t="n">
-        <v>53145</v>
+        <v>55239</v>
       </c>
       <c r="M45" t="n">
-        <v>11447</v>
+        <v>11765</v>
       </c>
       <c r="N45" t="n">
-        <v>41698</v>
+        <v>43474</v>
       </c>
     </row>
     <row r="46">
@@ -2471,13 +2471,13 @@
         <v>66503</v>
       </c>
       <c r="L46" t="n">
-        <v>68482</v>
+        <v>70781</v>
       </c>
       <c r="M46" t="n">
-        <v>11829</v>
+        <v>12157</v>
       </c>
       <c r="N46" t="n">
-        <v>56653</v>
+        <v>58624</v>
       </c>
     </row>
     <row r="47">
@@ -2515,13 +2515,13 @@
         <v>286539</v>
       </c>
       <c r="L47" t="n">
-        <v>135411</v>
+        <v>140410</v>
       </c>
       <c r="M47" t="n">
-        <v>57467</v>
+        <v>58595</v>
       </c>
       <c r="N47" t="n">
-        <v>77944</v>
+        <v>81815</v>
       </c>
     </row>
     <row r="48">
@@ -2559,13 +2559,13 @@
         <v>262442</v>
       </c>
       <c r="L48" t="n">
-        <v>135702</v>
+        <v>140729</v>
       </c>
       <c r="M48" t="n">
-        <v>56765</v>
+        <v>58059</v>
       </c>
       <c r="N48" t="n">
-        <v>78937</v>
+        <v>82670</v>
       </c>
     </row>
     <row r="49">
@@ -2603,13 +2603,13 @@
         <v>73813</v>
       </c>
       <c r="L49" t="n">
-        <v>50794</v>
+        <v>52505</v>
       </c>
       <c r="M49" t="n">
-        <v>15564</v>
+        <v>15890</v>
       </c>
       <c r="N49" t="n">
-        <v>35230</v>
+        <v>36615</v>
       </c>
     </row>
     <row r="50">
@@ -2647,13 +2647,13 @@
         <v>14115</v>
       </c>
       <c r="L50" t="n">
-        <v>42332</v>
+        <v>43502</v>
       </c>
       <c r="M50" t="n">
-        <v>5600</v>
+        <v>5745</v>
       </c>
       <c r="N50" t="n">
-        <v>36732</v>
+        <v>37757</v>
       </c>
     </row>
     <row r="51">
@@ -2691,13 +2691,13 @@
         <v>14887</v>
       </c>
       <c r="L51" t="n">
-        <v>21152</v>
+        <v>21744</v>
       </c>
       <c r="M51" t="n">
-        <v>4869</v>
+        <v>4996</v>
       </c>
       <c r="N51" t="n">
-        <v>16283</v>
+        <v>16748</v>
       </c>
     </row>
     <row r="52">
@@ -2735,13 +2735,13 @@
         <v>52222</v>
       </c>
       <c r="L52" t="n">
-        <v>50713</v>
+        <v>52384</v>
       </c>
       <c r="M52" t="n">
-        <v>13228</v>
+        <v>13576</v>
       </c>
       <c r="N52" t="n">
-        <v>37485</v>
+        <v>38808</v>
       </c>
     </row>
     <row r="53">
@@ -2779,13 +2779,13 @@
         <v>29739</v>
       </c>
       <c r="L53" t="n">
-        <v>37039</v>
+        <v>37819</v>
       </c>
       <c r="M53" t="n">
-        <v>9553</v>
+        <v>9752</v>
       </c>
       <c r="N53" t="n">
-        <v>27486</v>
+        <v>28067</v>
       </c>
     </row>
     <row r="54">
@@ -2823,13 +2823,13 @@
         <v>33755</v>
       </c>
       <c r="L54" t="n">
-        <v>33217</v>
+        <v>34891</v>
       </c>
       <c r="M54" t="n">
-        <v>8390</v>
+        <v>8727</v>
       </c>
       <c r="N54" t="n">
-        <v>24827</v>
+        <v>26164</v>
       </c>
     </row>
     <row r="55">
@@ -2867,13 +2867,13 @@
         <v>15489</v>
       </c>
       <c r="L55" t="n">
-        <v>12106</v>
+        <v>12978</v>
       </c>
       <c r="M55" t="n">
-        <v>3159</v>
+        <v>3418</v>
       </c>
       <c r="N55" t="n">
-        <v>8947</v>
+        <v>9560</v>
       </c>
     </row>
     <row r="56">
@@ -2911,13 +2911,13 @@
         <v>90057</v>
       </c>
       <c r="L56" t="n">
-        <v>67007</v>
+        <v>69044</v>
       </c>
       <c r="M56" t="n">
-        <v>16695</v>
+        <v>17163</v>
       </c>
       <c r="N56" t="n">
-        <v>50312</v>
+        <v>51881</v>
       </c>
     </row>
     <row r="57">
@@ -2955,13 +2955,13 @@
         <v>22869</v>
       </c>
       <c r="L57" t="n">
-        <v>24060</v>
+        <v>25340</v>
       </c>
       <c r="M57" t="n">
-        <v>5453</v>
+        <v>5688</v>
       </c>
       <c r="N57" t="n">
-        <v>18607</v>
+        <v>19652</v>
       </c>
     </row>
     <row r="58">
@@ -2999,13 +2999,13 @@
         <v>50900</v>
       </c>
       <c r="L58" t="n">
-        <v>76964</v>
+        <v>79658</v>
       </c>
       <c r="M58" t="n">
-        <v>15674</v>
+        <v>16252</v>
       </c>
       <c r="N58" t="n">
-        <v>61290</v>
+        <v>63406</v>
       </c>
     </row>
     <row r="59">
@@ -3043,13 +3043,13 @@
         <v>57445</v>
       </c>
       <c r="L59" t="n">
-        <v>44550</v>
+        <v>46292</v>
       </c>
       <c r="M59" t="n">
-        <v>12846</v>
+        <v>13229</v>
       </c>
       <c r="N59" t="n">
-        <v>31704</v>
+        <v>33063</v>
       </c>
     </row>
     <row r="60">
@@ -3087,13 +3087,13 @@
         <v>64646</v>
       </c>
       <c r="L60" t="n">
-        <v>75713</v>
+        <v>78332</v>
       </c>
       <c r="M60" t="n">
-        <v>22551</v>
+        <v>23220</v>
       </c>
       <c r="N60" t="n">
-        <v>53162</v>
+        <v>55112</v>
       </c>
     </row>
     <row r="61">
@@ -3131,13 +3131,13 @@
         <v>29176</v>
       </c>
       <c r="L61" t="n">
-        <v>25353</v>
+        <v>26506</v>
       </c>
       <c r="M61" t="n">
-        <v>6442</v>
+        <v>6683</v>
       </c>
       <c r="N61" t="n">
-        <v>18911</v>
+        <v>19823</v>
       </c>
     </row>
     <row r="62">
@@ -3175,13 +3175,13 @@
         <v>25083</v>
       </c>
       <c r="L62" t="n">
-        <v>44225</v>
+        <v>45221</v>
       </c>
       <c r="M62" t="n">
-        <v>6509</v>
+        <v>6672</v>
       </c>
       <c r="N62" t="n">
-        <v>37716</v>
+        <v>38549</v>
       </c>
     </row>
     <row r="63">
@@ -3219,13 +3219,13 @@
         <v>20109</v>
       </c>
       <c r="L63" t="n">
-        <v>25224</v>
+        <v>26589</v>
       </c>
       <c r="M63" t="n">
-        <v>3742</v>
+        <v>3864</v>
       </c>
       <c r="N63" t="n">
-        <v>21482</v>
+        <v>22725</v>
       </c>
     </row>
     <row r="64">
@@ -3263,13 +3263,13 @@
         <v>35709</v>
       </c>
       <c r="L64" t="n">
-        <v>25937</v>
+        <v>26935</v>
       </c>
       <c r="M64" t="n">
-        <v>4744</v>
+        <v>4922</v>
       </c>
       <c r="N64" t="n">
-        <v>21193</v>
+        <v>22013</v>
       </c>
     </row>
     <row r="65">
@@ -3307,13 +3307,13 @@
         <v>69002</v>
       </c>
       <c r="L65" t="n">
-        <v>52376</v>
+        <v>54447</v>
       </c>
       <c r="M65" t="n">
-        <v>10999</v>
+        <v>11380</v>
       </c>
       <c r="N65" t="n">
-        <v>41377</v>
+        <v>43067</v>
       </c>
     </row>
     <row r="66">
@@ -3351,13 +3351,13 @@
         <v>85499</v>
       </c>
       <c r="L66" t="n">
-        <v>55387</v>
+        <v>57565</v>
       </c>
       <c r="M66" t="n">
-        <v>11296</v>
+        <v>11579</v>
       </c>
       <c r="N66" t="n">
-        <v>44091</v>
+        <v>45986</v>
       </c>
     </row>
     <row r="67">
@@ -3395,13 +3395,13 @@
         <v>27583</v>
       </c>
       <c r="L67" t="n">
-        <v>40684</v>
+        <v>41532</v>
       </c>
       <c r="M67" t="n">
-        <v>12525</v>
+        <v>12760</v>
       </c>
       <c r="N67" t="n">
-        <v>28159</v>
+        <v>28772</v>
       </c>
     </row>
     <row r="68">
@@ -3439,13 +3439,13 @@
         <v>42869</v>
       </c>
       <c r="L68" t="n">
-        <v>40993</v>
+        <v>42400</v>
       </c>
       <c r="M68" t="n">
-        <v>8713</v>
+        <v>9064</v>
       </c>
       <c r="N68" t="n">
-        <v>32280</v>
+        <v>33336</v>
       </c>
     </row>
     <row r="69">
@@ -3483,13 +3483,13 @@
         <v>78610</v>
       </c>
       <c r="L69" t="n">
-        <v>58355</v>
+        <v>60845</v>
       </c>
       <c r="M69" t="n">
-        <v>9756</v>
+        <v>10127</v>
       </c>
       <c r="N69" t="n">
-        <v>48599</v>
+        <v>50718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>